<commit_message>
Changed schedule 5 hours behind
</commit_message>
<xml_diff>
--- a/automated_message/schedule.xlsx
+++ b/automated_message/schedule.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
   <si>
     <t>name</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>opening ceremonies</t>
+  </si>
+  <si>
+    <t>5:00</t>
   </si>
   <si>
     <t>PGCLL 127</t>
@@ -536,7 +539,7 @@
         <v>46039</v>
       </c>
       <c r="C2" s="3">
-        <v>1.375</v>
+        <v>46023.166666666664</v>
       </c>
       <c r="D2" s="4">
         <v>30</v>
@@ -552,354 +555,354 @@
       <c r="B3" s="2">
         <v>46039</v>
       </c>
-      <c r="C3" s="5">
-        <v>1.4166666666666667</v>
+      <c r="C3" s="5" t="s">
+        <v>8</v>
       </c>
       <c r="D3" s="6">
         <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2">
         <v>46039</v>
       </c>
       <c r="C4" s="3">
-        <v>46023.458333333336</v>
+        <v>46023.291666666664</v>
       </c>
       <c r="D4" s="4">
         <v>30</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2">
         <v>46039</v>
       </c>
       <c r="C5" s="3">
-        <v>1.5416666666666665</v>
+        <v>46023.333333333336</v>
       </c>
       <c r="D5" s="4">
         <v>20</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="2">
         <v>46039</v>
       </c>
       <c r="C6" s="3">
-        <v>1.5833333333333335</v>
+        <v>46023.375</v>
       </c>
       <c r="D6" s="4">
         <v>15</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2">
         <v>46039</v>
       </c>
       <c r="C7" s="3">
-        <v>1.6041666666666665</v>
+        <v>46023.395833333336</v>
       </c>
       <c r="D7" s="4">
         <v>20</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2">
         <v>46039</v>
       </c>
       <c r="C8" s="3">
-        <v>1.625</v>
+        <v>46023.416666666664</v>
       </c>
       <c r="D8" s="4">
         <v>30</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9" s="2">
         <v>46039</v>
       </c>
       <c r="C9" s="3">
-        <v>1.7083333333333335</v>
+        <v>46023</v>
       </c>
       <c r="D9" s="4">
         <v>20</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10" s="2">
         <v>46039</v>
       </c>
       <c r="C10" s="3">
-        <v>1.7291666666666665</v>
+        <v>46023.020833333336</v>
       </c>
       <c r="D10" s="4">
         <v>20</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B11" s="2">
         <v>46039</v>
       </c>
       <c r="C11" s="3">
-        <v>1.75</v>
+        <v>46023.541666666664</v>
       </c>
       <c r="D11" s="4">
         <v>30</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B12" s="2">
         <v>46039</v>
       </c>
       <c r="C12" s="3">
-        <v>1.7916666666666665</v>
+        <v>46023.583333333336</v>
       </c>
       <c r="D12" s="4">
         <v>20</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B13" s="2">
         <v>46039</v>
       </c>
       <c r="C13" s="3">
-        <v>1.8333333333333335</v>
+        <v>46023.625</v>
       </c>
       <c r="D13" s="4">
         <v>20</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B14" s="2">
         <v>46039</v>
       </c>
       <c r="C14" s="3">
-        <v>1.875</v>
+        <v>46023.666666666664</v>
       </c>
       <c r="D14" s="4">
         <v>20</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15" s="2">
         <v>46039</v>
       </c>
       <c r="C15" s="3">
-        <v>1.8958333333333335</v>
+        <v>46023.6875</v>
       </c>
       <c r="D15" s="4">
         <v>20</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B16" s="2">
         <v>46039</v>
       </c>
       <c r="C16" s="3">
-        <v>1.9583333333333335</v>
+        <v>46023.75</v>
       </c>
       <c r="D16" s="4">
         <v>15</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B17" s="2">
         <v>46039</v>
       </c>
       <c r="C17" s="3">
-        <v>1.9583333333333335</v>
+        <v>46023.75</v>
       </c>
       <c r="D17" s="4">
         <v>30</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2">
-        <v>46040</v>
+        <v>46039</v>
       </c>
       <c r="C18" s="3">
-        <v>1.0833333333333333</v>
+        <v>46023.875</v>
       </c>
       <c r="D18" s="4">
         <v>30</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B19" s="2">
         <v>46040</v>
       </c>
       <c r="C19" s="3">
-        <v>1.3333333333333333</v>
+        <v>46023.125</v>
       </c>
       <c r="D19" s="4">
         <v>30</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B20" s="2">
         <v>46040</v>
       </c>
       <c r="C20" s="3">
-        <v>1.4791666666666667</v>
+        <v>46023.270833333336</v>
       </c>
       <c r="D20" s="4">
         <v>30</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21" s="2">
         <v>46040</v>
       </c>
       <c r="C21" s="3">
-        <v>1.5</v>
+        <v>46023.291666666664</v>
       </c>
       <c r="D21" s="4">
         <v>20</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B22" s="2">
         <v>46040</v>
       </c>
       <c r="C22" s="3">
-        <v>1.5416666666666665</v>
+        <v>46023.333333333336</v>
       </c>
       <c r="D22" s="4">
         <v>20</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23" s="2">
         <v>46040</v>
       </c>
       <c r="C23" s="3">
-        <v>1.6875</v>
+        <v>46023.479166666664</v>
       </c>
       <c r="D23" s="4">
         <v>20</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made schedule 5 hours ahead
</commit_message>
<xml_diff>
--- a/automated_message/schedule.xlsx
+++ b/automated_message/schedule.xlsx
@@ -40,7 +40,7 @@
     <t>opening ceremonies</t>
   </si>
   <si>
-    <t>5:00</t>
+    <t>14:00</t>
   </si>
   <si>
     <t>PGCLL 127</t>
@@ -539,7 +539,7 @@
         <v>46039</v>
       </c>
       <c r="C2" s="3">
-        <v>46023.166666666664</v>
+        <v>46023.583333333336</v>
       </c>
       <c r="D2" s="4">
         <v>30</v>
@@ -573,7 +573,7 @@
         <v>46039</v>
       </c>
       <c r="C4" s="3">
-        <v>46023.291666666664</v>
+        <v>46023.708333333336</v>
       </c>
       <c r="D4" s="4">
         <v>30</v>
@@ -590,7 +590,7 @@
         <v>46039</v>
       </c>
       <c r="C5" s="3">
-        <v>46023.333333333336</v>
+        <v>46023.75</v>
       </c>
       <c r="D5" s="4">
         <v>20</v>
@@ -607,7 +607,7 @@
         <v>46039</v>
       </c>
       <c r="C6" s="3">
-        <v>46023.375</v>
+        <v>46023.791666666664</v>
       </c>
       <c r="D6" s="4">
         <v>15</v>
@@ -624,7 +624,7 @@
         <v>46039</v>
       </c>
       <c r="C7" s="3">
-        <v>46023.395833333336</v>
+        <v>46023.8125</v>
       </c>
       <c r="D7" s="4">
         <v>20</v>
@@ -641,7 +641,7 @@
         <v>46039</v>
       </c>
       <c r="C8" s="3">
-        <v>46023.416666666664</v>
+        <v>46023.833333333336</v>
       </c>
       <c r="D8" s="4">
         <v>30</v>
@@ -658,7 +658,7 @@
         <v>46039</v>
       </c>
       <c r="C9" s="3">
-        <v>46023</v>
+        <v>46023.916666666664</v>
       </c>
       <c r="D9" s="4">
         <v>20</v>
@@ -675,7 +675,7 @@
         <v>46039</v>
       </c>
       <c r="C10" s="3">
-        <v>46023.020833333336</v>
+        <v>46023.9375</v>
       </c>
       <c r="D10" s="4">
         <v>20</v>
@@ -692,7 +692,7 @@
         <v>46039</v>
       </c>
       <c r="C11" s="3">
-        <v>46023.541666666664</v>
+        <v>46023.958333333336</v>
       </c>
       <c r="D11" s="4">
         <v>30</v>
@@ -706,10 +706,10 @@
         <v>22</v>
       </c>
       <c r="B12" s="2">
-        <v>46039</v>
+        <v>46040</v>
       </c>
       <c r="C12" s="3">
-        <v>46023.583333333336</v>
+        <v>46023</v>
       </c>
       <c r="D12" s="4">
         <v>20</v>
@@ -723,10 +723,10 @@
         <v>23</v>
       </c>
       <c r="B13" s="2">
-        <v>46039</v>
+        <v>46040</v>
       </c>
       <c r="C13" s="3">
-        <v>46023.625</v>
+        <v>46023.041666666664</v>
       </c>
       <c r="D13" s="4">
         <v>20</v>
@@ -740,10 +740,10 @@
         <v>24</v>
       </c>
       <c r="B14" s="2">
-        <v>46039</v>
+        <v>46040</v>
       </c>
       <c r="C14" s="3">
-        <v>46023.666666666664</v>
+        <v>46023.083333333336</v>
       </c>
       <c r="D14" s="4">
         <v>20</v>
@@ -757,10 +757,10 @@
         <v>25</v>
       </c>
       <c r="B15" s="2">
-        <v>46039</v>
+        <v>46040</v>
       </c>
       <c r="C15" s="3">
-        <v>46023.6875</v>
+        <v>46023.104166666664</v>
       </c>
       <c r="D15" s="4">
         <v>20</v>
@@ -774,10 +774,10 @@
         <v>26</v>
       </c>
       <c r="B16" s="2">
-        <v>46039</v>
+        <v>46040</v>
       </c>
       <c r="C16" s="3">
-        <v>46023.75</v>
+        <v>46023.166666666664</v>
       </c>
       <c r="D16" s="4">
         <v>15</v>
@@ -791,10 +791,10 @@
         <v>27</v>
       </c>
       <c r="B17" s="2">
-        <v>46039</v>
+        <v>46040</v>
       </c>
       <c r="C17" s="3">
-        <v>46023.75</v>
+        <v>46023.166666666664</v>
       </c>
       <c r="D17" s="4">
         <v>30</v>
@@ -808,10 +808,10 @@
         <v>29</v>
       </c>
       <c r="B18" s="2">
-        <v>46039</v>
+        <v>46040</v>
       </c>
       <c r="C18" s="3">
-        <v>46023.875</v>
+        <v>46023.291666666664</v>
       </c>
       <c r="D18" s="4">
         <v>30</v>
@@ -828,7 +828,7 @@
         <v>46040</v>
       </c>
       <c r="C19" s="3">
-        <v>46023.125</v>
+        <v>46023.541666666664</v>
       </c>
       <c r="D19" s="4">
         <v>30</v>
@@ -845,7 +845,7 @@
         <v>46040</v>
       </c>
       <c r="C20" s="3">
-        <v>46023.270833333336</v>
+        <v>46023.6875</v>
       </c>
       <c r="D20" s="4">
         <v>30</v>
@@ -862,7 +862,7 @@
         <v>46040</v>
       </c>
       <c r="C21" s="3">
-        <v>46023.291666666664</v>
+        <v>46023.708333333336</v>
       </c>
       <c r="D21" s="4">
         <v>20</v>
@@ -879,7 +879,7 @@
         <v>46040</v>
       </c>
       <c r="C22" s="3">
-        <v>46023.333333333336</v>
+        <v>46023.75</v>
       </c>
       <c r="D22" s="4">
         <v>20</v>
@@ -896,7 +896,7 @@
         <v>46040</v>
       </c>
       <c r="C23" s="3">
-        <v>46023.479166666664</v>
+        <v>46023.895833333336</v>
       </c>
       <c r="D23" s="4">
         <v>20</v>

</xml_diff>